<commit_message>
Forms sync auto batch 2: 5000 files
</commit_message>
<xml_diff>
--- a/counselor_forms/020_dating_survey--counselor_forms.xlsx
+++ b/counselor_forms/020_dating_survey--counselor_forms.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1102,8 +1102,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'value':_'single',_'label':_'single'}</t>
+          <t>single</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'value': 'Single', 'label': 'Single'}</t>
+          <t>Single</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1148,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'value':_'in_a_relationship',_'label':_'in_a_relationship'}</t>
+          <t>in_a_relationship</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'value': 'In a relationship', 'label': 'In a relationship'}</t>
+          <t>In a relationship</t>
         </is>
       </c>
     </row>
@@ -1165,12 +1165,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{'value':_'in_a_long-term_relationship',_'label':_'in_a_long-term_relationship'}</t>
+          <t>in_a_long-term_relationship</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'value': 'In a long-term relationship', 'label': 'In a long-term relationship'}</t>
+          <t>In a long-term relationship</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{'value':_'in_a_marriage',_'label':_'in_a_marriage'}</t>
+          <t>in_a_marriage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{'value': 'In a marriage', 'label': 'In a marriage'}</t>
+          <t>In a marriage</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -1216,12 +1216,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{'value':_'online',_'label':_'online'}</t>
+          <t>online</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{'value': 'Online', 'label': 'Online'}</t>
+          <t>Online</t>
         </is>
       </c>
     </row>
@@ -1233,12 +1233,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{'value':_'mutual_friend',_'label':_'mutual_friend'}</t>
+          <t>mutual_friend</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>{'value': 'Mutual friend', 'label': 'Mutual friend'}</t>
+          <t>Mutual friend</t>
         </is>
       </c>
     </row>
@@ -1250,12 +1250,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{'value':_'social_media',_'label':_'social_media'}</t>
+          <t>social_media</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>{'value': 'Social media', 'label': 'Social media'}</t>
+          <t>Social media</t>
         </is>
       </c>
     </row>
@@ -1267,12 +1267,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{'value':_'through_a_friend_of_a_friend',_'label':_'through_a_friend_of_a_friend'}</t>
+          <t>through_a_friend_of_a_friend</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{'value': 'Through a friend of a friend', 'label': 'Through a friend of a friend'}</t>
+          <t>Through a friend of a friend</t>
         </is>
       </c>
     </row>
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'value':_'at_an_event',_'label':_'at_an_event'}</t>
+          <t>at_an_event</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>{'value': 'At an event', 'label': 'At an event'}</t>
+          <t>At an event</t>
         </is>
       </c>
     </row>
@@ -1301,12 +1301,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -1318,12 +1318,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'value':_'talked_on_the_phone',_'label':_'talked_on_the_phone'}</t>
+          <t>talked_on_the_phone</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>{'value': 'Talked on the phone', 'label': 'Talked on the phone'}</t>
+          <t>Talked on the phone</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1335,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{'value':_'sent_a_text_message',_'label':_'sent_a_text_message'}</t>
+          <t>sent_a_text_message</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{'value': 'Sent a text message', 'label': 'Sent a text message'}</t>
+          <t>Sent a text message</t>
         </is>
       </c>
     </row>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{'value':_'sent_a_message_online',_'label':_'sent_a_message_online'}</t>
+          <t>sent_a_message_online</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>{'value': 'Sent a message online', 'label': 'Sent a message online'}</t>
+          <t>Sent a message online</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{'value':_'sent_an_email',_'label':_'sent_an_email'}</t>
+          <t>sent_an_email</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>{'value': 'Sent an email', 'label': 'Sent an email'}</t>
+          <t>Sent an email</t>
         </is>
       </c>
     </row>
@@ -1386,12 +1386,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>{'value':_'fun_and_casual',_'label':_'fun_and_casual'}</t>
+          <t>fun_and_casual</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>{'value': 'Fun and casual', 'label': 'Fun and casual'}</t>
+          <t>Fun and casual</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{'value':_'romantic',_'label':_'romantic'}</t>
+          <t>romantic</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>{'value': 'Romantic', 'label': 'Romantic'}</t>
+          <t>Romantic</t>
         </is>
       </c>
     </row>
@@ -1437,12 +1437,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>{'value':_'friendship',_'label':_'friendship'}</t>
+          <t>friendship</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>{'value': 'Friendship', 'label': 'Friendship'}</t>
+          <t>Friendship</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1471,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>{'value':_'a_few_hours',_'label':_'a_few_hours'}</t>
+          <t>a_few_hours</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{'value': 'A few hours', 'label': 'A few hours'}</t>
+          <t>A few hours</t>
         </is>
       </c>
     </row>
@@ -1488,12 +1488,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>{'value':_'a_few_days',_'label':_'a_few_days'}</t>
+          <t>a_few_days</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>{'value': 'A few days', 'label': 'A few days'}</t>
+          <t>A few days</t>
         </is>
       </c>
     </row>
@@ -1505,12 +1505,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{'value':_'a_few_weeks',_'label':_'a_few_weeks'}</t>
+          <t>a_few_weeks</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{'value': 'A few weeks', 'label': 'A few weeks'}</t>
+          <t>A few weeks</t>
         </is>
       </c>
     </row>
@@ -1522,12 +1522,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{'value':_'a_few_months',_'label':_'a_few_months'}</t>
+          <t>a_few_months</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{'value': 'A few months', 'label': 'A few months'}</t>
+          <t>A few months</t>
         </is>
       </c>
     </row>
@@ -1539,12 +1539,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>{'value':_'less_than_a_week',_'label':_'less_than_a_week'}</t>
+          <t>less_than_a_week</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{'value': 'Less than a week', 'label': 'Less than a week'}</t>
+          <t>Less than a week</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>{'value':_'more_than_a_month',_'label':_'more_than_a_month'}</t>
+          <t>more_than_a_month</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>{'value': 'More than a month', 'label': 'More than a month'}</t>
+          <t>More than a month</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1573,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>{'value':_'hobbies',_'label':_'hobbies'}</t>
+          <t>hobbies</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{'value': 'Hobbies', 'label': 'Hobbies'}</t>
+          <t>Hobbies</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>{'value':_'hiking',_'label':_'hiking'}</t>
+          <t>hiking</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>{'value': 'Hiking', 'label': 'Hiking'}</t>
+          <t>Hiking</t>
         </is>
       </c>
     </row>
@@ -1624,12 +1624,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>{'value':_'movies',_'label':_'movies'}</t>
+          <t>movies</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>{'value': 'Movies', 'label': 'Movies'}</t>
+          <t>Movies</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1641,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>{'value':_'reading',_'label':_'reading'}</t>
+          <t>reading</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>{'value': 'Reading', 'label': 'Reading'}</t>
+          <t>Reading</t>
         </is>
       </c>
     </row>
@@ -1658,12 +1658,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>{'value':_'traveling',_'label':_'traveling'}</t>
+          <t>traveling</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>{'value': 'Traveling', 'label': 'Traveling'}</t>
+          <t>Traveling</t>
         </is>
       </c>
     </row>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -1692,12 +1692,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>{'value':_'a_lot',_'label':_'a_lot'}</t>
+          <t>a_lot</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>{'value': 'A lot', 'label': 'A lot'}</t>
+          <t>A lot</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>{'value':_'somewhat',_'label':_'somewhat'}</t>
+          <t>somewhat</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>{'value': 'Somewhat', 'label': 'Somewhat'}</t>
+          <t>Somewhat</t>
         </is>
       </c>
     </row>
@@ -1726,12 +1726,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>{'value':_'not_very_much',_'label':_'not_very_much'}</t>
+          <t>not_very_much</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>{'value': 'Not very much', 'label': 'Not very much'}</t>
+          <t>Not very much</t>
         </is>
       </c>
     </row>
@@ -1743,12 +1743,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>{'value':_'not_at_all',_'label':_'not_at_all'}</t>
+          <t>not_at_all</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>{'value': 'Not at all', 'label': 'Not at all'}</t>
+          <t>Not at all</t>
         </is>
       </c>
     </row>
@@ -1760,12 +1760,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1777,12 +1777,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1794,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1828,12 +1828,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1862,12 +1862,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1879,12 +1879,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>{'value':_'happy',_'label':_'happy'}</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>{'value': 'Happy', 'label': 'Happy'}</t>
+          <t>Happy</t>
         </is>
       </c>
     </row>
@@ -1947,12 +1947,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>{'value':_'sad',_'label':_'sad'}</t>
+          <t>sad</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>{'value': 'Sad', 'label': 'Sad'}</t>
+          <t>Sad</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>{'value':_'excited',_'label':_'excited'}</t>
+          <t>excited</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>{'value': 'Excited', 'label': 'Excited'}</t>
+          <t>Excited</t>
         </is>
       </c>
     </row>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>{'value':_'bored',_'label':_'bored'}</t>
+          <t>bored</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>{'value': 'Bored', 'label': 'Bored'}</t>
+          <t>Bored</t>
         </is>
       </c>
     </row>
@@ -1998,12 +1998,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>{'value':_'other',_'label':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>{'value': 'Other', 'label': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -2032,12 +2032,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -2049,12 +2049,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -2083,12 +2083,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>{'value':_1,_'label':_1}</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>{'value': 1, 'label': 1}</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>{'value':_2,_'label':_2}</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>{'value': 2, 'label': 2}</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2117,12 +2117,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>{'value':_3,_'label':_3}</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>{'value': 3, 'label': 3}</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2134,12 +2134,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>{'value':_4,_'label':_4}</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>{'value': 4, 'label': 4}</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2151,12 +2151,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>{'value':_5,_'label':_5}</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>{'value': 5, 'label': 5}</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -2168,12 +2168,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>{'value':_true,_'label':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>{'value': True, 'label': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -2185,12 +2185,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>{'value':_false,_'label':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>{'value': False, 'label': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>

</xml_diff>